<commit_message>
feat: add Dockerfile, docker-compose, resume integration, and github actions for auto-deployment
</commit_message>
<xml_diff>
--- a/ระบบส่วนงานของฟอร์ด.xlsx
+++ b/ระบบส่วนงานของฟอร์ด.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dx_de\OneDrive\Desktop\งาน  Ford ทั้งหมด\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dx_de\OneDrive\Desktop\ผลลงาน Port forlio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4E63DB3-DBF6-4BDB-92BE-E0CF47464E7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E55C1643-B18B-4FDA-B5C1-4DABB3ECA24A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C480879D-218D-4E6B-964A-85EB4AF78C11}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="58">
   <si>
     <t>Low</t>
   </si>
@@ -208,6 +208,12 @@
   </si>
   <si>
     <t>4 วัน</t>
+  </si>
+  <si>
+    <t>จัดทำ Haco Nexus</t>
+  </si>
+  <si>
+    <t>Hold</t>
   </si>
 </sst>
 </file>
@@ -290,7 +296,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -339,6 +345,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="12">
     <border>
@@ -493,7 +505,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -543,28 +555,74 @@
     <xf numFmtId="9" fontId="7" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="2" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -588,52 +646,13 @@
     <xf numFmtId="164" fontId="7" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="9" fontId="7" fillId="9" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="ปกติ" xfId="0" builtinId="0"/>
@@ -968,7 +987,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D86B0126-D6EA-41B8-876E-8FCB1435C707}">
-  <dimension ref="A1:M26"/>
+  <dimension ref="A1:M27"/>
   <sheetFormatPr defaultRowHeight="16.8" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="5.8984375" bestFit="1" customWidth="1"/>
@@ -986,100 +1005,100 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.4">
-      <c r="A1" s="39" t="s">
+      <c r="A1" s="19" t="s">
         <v>29</v>
       </c>
-      <c r="B1" s="39"/>
-      <c r="C1" s="39"/>
-      <c r="D1" s="39"/>
-      <c r="E1" s="39"/>
-      <c r="F1" s="39"/>
-      <c r="G1" s="39"/>
-      <c r="H1" s="39"/>
-      <c r="I1" s="39"/>
-      <c r="J1" s="39"/>
-      <c r="K1" s="39"/>
-      <c r="L1" s="39"/>
-      <c r="M1" s="39"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
+      <c r="K1" s="19"/>
+      <c r="L1" s="19"/>
+      <c r="M1" s="19"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.4">
-      <c r="A2" s="39"/>
-      <c r="B2" s="39"/>
-      <c r="C2" s="39"/>
-      <c r="D2" s="39"/>
-      <c r="E2" s="39"/>
-      <c r="F2" s="39"/>
-      <c r="G2" s="39"/>
-      <c r="H2" s="39"/>
-      <c r="I2" s="39"/>
-      <c r="J2" s="39"/>
-      <c r="K2" s="39"/>
-      <c r="L2" s="39"/>
-      <c r="M2" s="39"/>
+      <c r="A2" s="19"/>
+      <c r="B2" s="19"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
+      <c r="H2" s="19"/>
+      <c r="I2" s="19"/>
+      <c r="J2" s="19"/>
+      <c r="K2" s="19"/>
+      <c r="L2" s="19"/>
+      <c r="M2" s="19"/>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.4">
-      <c r="A3" s="39"/>
-      <c r="B3" s="39"/>
-      <c r="C3" s="39"/>
-      <c r="D3" s="39"/>
-      <c r="E3" s="39"/>
-      <c r="F3" s="39"/>
-      <c r="G3" s="39"/>
-      <c r="H3" s="39"/>
-      <c r="I3" s="39"/>
-      <c r="J3" s="39"/>
-      <c r="K3" s="39"/>
-      <c r="L3" s="39"/>
-      <c r="M3" s="39"/>
+      <c r="A3" s="19"/>
+      <c r="B3" s="19"/>
+      <c r="C3" s="19"/>
+      <c r="D3" s="19"/>
+      <c r="E3" s="19"/>
+      <c r="F3" s="19"/>
+      <c r="G3" s="19"/>
+      <c r="H3" s="19"/>
+      <c r="I3" s="19"/>
+      <c r="J3" s="19"/>
+      <c r="K3" s="19"/>
+      <c r="L3" s="19"/>
+      <c r="M3" s="19"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.4">
-      <c r="A4" s="39"/>
-      <c r="B4" s="39"/>
-      <c r="C4" s="39"/>
-      <c r="D4" s="39"/>
-      <c r="E4" s="39"/>
-      <c r="F4" s="39"/>
-      <c r="G4" s="39"/>
-      <c r="H4" s="39"/>
-      <c r="I4" s="39"/>
-      <c r="J4" s="39"/>
-      <c r="K4" s="39"/>
-      <c r="L4" s="39"/>
-      <c r="M4" s="39"/>
+      <c r="A4" s="19"/>
+      <c r="B4" s="19"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="19"/>
+      <c r="F4" s="19"/>
+      <c r="G4" s="19"/>
+      <c r="H4" s="19"/>
+      <c r="I4" s="19"/>
+      <c r="J4" s="19"/>
+      <c r="K4" s="19"/>
+      <c r="L4" s="19"/>
+      <c r="M4" s="19"/>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.4">
-      <c r="A5" s="39"/>
-      <c r="B5" s="39"/>
-      <c r="C5" s="39"/>
-      <c r="D5" s="39"/>
-      <c r="E5" s="39"/>
-      <c r="F5" s="39"/>
-      <c r="G5" s="39"/>
-      <c r="H5" s="39"/>
-      <c r="I5" s="39"/>
-      <c r="J5" s="39"/>
-      <c r="K5" s="39"/>
-      <c r="L5" s="39"/>
-      <c r="M5" s="39"/>
+      <c r="A5" s="19"/>
+      <c r="B5" s="19"/>
+      <c r="C5" s="19"/>
+      <c r="D5" s="19"/>
+      <c r="E5" s="19"/>
+      <c r="F5" s="19"/>
+      <c r="G5" s="19"/>
+      <c r="H5" s="19"/>
+      <c r="I5" s="19"/>
+      <c r="J5" s="19"/>
+      <c r="K5" s="19"/>
+      <c r="L5" s="19"/>
+      <c r="M5" s="19"/>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.4">
-      <c r="A6" s="40" t="s">
+      <c r="A6" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="41"/>
-      <c r="C6" s="41"/>
-      <c r="D6" s="41"/>
-      <c r="E6" s="41"/>
-      <c r="F6" s="41"/>
-      <c r="G6" s="41"/>
-      <c r="H6" s="41"/>
-      <c r="I6" s="41"/>
-      <c r="J6" s="42"/>
-      <c r="K6" s="43" t="s">
+      <c r="B6" s="21"/>
+      <c r="C6" s="21"/>
+      <c r="D6" s="21"/>
+      <c r="E6" s="21"/>
+      <c r="F6" s="21"/>
+      <c r="G6" s="21"/>
+      <c r="H6" s="21"/>
+      <c r="I6" s="21"/>
+      <c r="J6" s="22"/>
+      <c r="K6" s="23" t="s">
         <v>15</v>
       </c>
-      <c r="L6" s="44"/>
-      <c r="M6" s="45"/>
+      <c r="L6" s="24"/>
+      <c r="M6" s="25"/>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A7" s="1" t="s">
@@ -1123,350 +1142,350 @@
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.4">
-      <c r="A8" s="35">
+      <c r="A8" s="26">
         <v>1</v>
       </c>
-      <c r="B8" s="22" t="s">
+      <c r="B8" s="27" t="s">
         <v>38</v>
       </c>
-      <c r="C8" s="22" t="s">
+      <c r="C8" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="D8" s="22" t="s">
+      <c r="D8" s="27" t="s">
         <v>30</v>
       </c>
       <c r="E8" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="F8" s="22" t="s">
+      <c r="F8" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="G8" s="22" t="s">
+      <c r="G8" s="27" t="s">
         <v>5</v>
       </c>
       <c r="H8" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="I8" s="22" t="s">
+      <c r="I8" s="27" t="s">
         <v>7</v>
       </c>
-      <c r="J8" s="32" t="s">
+      <c r="J8" s="33" t="s">
         <v>8</v>
       </c>
-      <c r="K8" s="19">
+      <c r="K8" s="30">
         <v>244571</v>
       </c>
-      <c r="L8" s="19">
+      <c r="L8" s="30">
         <v>244574</v>
       </c>
-      <c r="M8" s="22" t="s">
+      <c r="M8" s="27" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.4">
-      <c r="A9" s="35"/>
-      <c r="B9" s="23"/>
-      <c r="C9" s="23"/>
-      <c r="D9" s="23"/>
+      <c r="A9" s="26"/>
+      <c r="B9" s="28"/>
+      <c r="C9" s="28"/>
+      <c r="D9" s="28"/>
       <c r="E9" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="F9" s="23"/>
-      <c r="G9" s="23"/>
+      <c r="F9" s="28"/>
+      <c r="G9" s="28"/>
       <c r="H9" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="I9" s="23"/>
-      <c r="J9" s="33"/>
-      <c r="K9" s="20"/>
-      <c r="L9" s="20"/>
-      <c r="M9" s="23"/>
+      <c r="I9" s="28"/>
+      <c r="J9" s="34"/>
+      <c r="K9" s="31"/>
+      <c r="L9" s="31"/>
+      <c r="M9" s="28"/>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.4">
-      <c r="A10" s="35"/>
-      <c r="B10" s="24"/>
-      <c r="C10" s="24"/>
-      <c r="D10" s="24"/>
+      <c r="A10" s="26"/>
+      <c r="B10" s="29"/>
+      <c r="C10" s="29"/>
+      <c r="D10" s="29"/>
       <c r="E10" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="F10" s="24"/>
-      <c r="G10" s="24"/>
+      <c r="F10" s="29"/>
+      <c r="G10" s="29"/>
       <c r="H10" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="I10" s="24"/>
-      <c r="J10" s="34"/>
-      <c r="K10" s="21"/>
-      <c r="L10" s="21"/>
-      <c r="M10" s="24"/>
+      <c r="I10" s="29"/>
+      <c r="J10" s="35"/>
+      <c r="K10" s="32"/>
+      <c r="L10" s="32"/>
+      <c r="M10" s="29"/>
     </row>
     <row r="11" spans="1:13" ht="16.8" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A11" s="35">
+      <c r="A11" s="26">
         <v>2</v>
       </c>
       <c r="B11" s="36" t="s">
         <v>39</v>
       </c>
-      <c r="C11" s="22" t="s">
+      <c r="C11" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="D11" s="22" t="s">
+      <c r="D11" s="27" t="s">
         <v>2</v>
       </c>
       <c r="E11" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="F11" s="22" t="s">
+      <c r="F11" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="G11" s="22" t="s">
+      <c r="G11" s="27" t="s">
         <v>5</v>
       </c>
       <c r="H11" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="I11" s="22" t="s">
+      <c r="I11" s="27" t="s">
         <v>7</v>
       </c>
-      <c r="J11" s="32" t="s">
+      <c r="J11" s="33" t="s">
         <v>8</v>
       </c>
-      <c r="K11" s="19">
+      <c r="K11" s="30">
         <v>244595</v>
       </c>
-      <c r="L11" s="19">
+      <c r="L11" s="30">
         <v>244610</v>
       </c>
-      <c r="M11" s="22" t="s">
+      <c r="M11" s="27" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.4">
-      <c r="A12" s="35"/>
+      <c r="A12" s="26"/>
       <c r="B12" s="37"/>
-      <c r="C12" s="23"/>
-      <c r="D12" s="23"/>
+      <c r="C12" s="28"/>
+      <c r="D12" s="28"/>
       <c r="E12" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="F12" s="23"/>
-      <c r="G12" s="23"/>
+      <c r="F12" s="28"/>
+      <c r="G12" s="28"/>
       <c r="H12" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="I12" s="23"/>
-      <c r="J12" s="33"/>
-      <c r="K12" s="20"/>
-      <c r="L12" s="20"/>
-      <c r="M12" s="23"/>
+      <c r="I12" s="28"/>
+      <c r="J12" s="34"/>
+      <c r="K12" s="31"/>
+      <c r="L12" s="31"/>
+      <c r="M12" s="28"/>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.4">
-      <c r="A13" s="35"/>
+      <c r="A13" s="26"/>
       <c r="B13" s="37"/>
-      <c r="C13" s="23"/>
-      <c r="D13" s="23"/>
+      <c r="C13" s="28"/>
+      <c r="D13" s="28"/>
       <c r="E13" s="5"/>
-      <c r="F13" s="23"/>
-      <c r="G13" s="23"/>
+      <c r="F13" s="28"/>
+      <c r="G13" s="28"/>
       <c r="H13" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="I13" s="23"/>
-      <c r="J13" s="33"/>
-      <c r="K13" s="20"/>
-      <c r="L13" s="20"/>
-      <c r="M13" s="23"/>
+      <c r="I13" s="28"/>
+      <c r="J13" s="34"/>
+      <c r="K13" s="31"/>
+      <c r="L13" s="31"/>
+      <c r="M13" s="28"/>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.4">
-      <c r="A14" s="35"/>
+      <c r="A14" s="26"/>
       <c r="B14" s="37"/>
-      <c r="C14" s="23"/>
-      <c r="D14" s="23"/>
+      <c r="C14" s="28"/>
+      <c r="D14" s="28"/>
       <c r="E14" s="5"/>
-      <c r="F14" s="23"/>
-      <c r="G14" s="23"/>
+      <c r="F14" s="28"/>
+      <c r="G14" s="28"/>
       <c r="H14" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="I14" s="23"/>
-      <c r="J14" s="33"/>
-      <c r="K14" s="20"/>
-      <c r="L14" s="20"/>
-      <c r="M14" s="23"/>
+      <c r="I14" s="28"/>
+      <c r="J14" s="34"/>
+      <c r="K14" s="31"/>
+      <c r="L14" s="31"/>
+      <c r="M14" s="28"/>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.4">
-      <c r="A15" s="35"/>
+      <c r="A15" s="26"/>
       <c r="B15" s="38"/>
-      <c r="C15" s="24"/>
-      <c r="D15" s="24"/>
+      <c r="C15" s="29"/>
+      <c r="D15" s="29"/>
       <c r="E15" s="5"/>
-      <c r="F15" s="24"/>
-      <c r="G15" s="24"/>
+      <c r="F15" s="29"/>
+      <c r="G15" s="29"/>
       <c r="H15" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="I15" s="24"/>
-      <c r="J15" s="34"/>
-      <c r="K15" s="21"/>
-      <c r="L15" s="21"/>
-      <c r="M15" s="24"/>
+      <c r="I15" s="29"/>
+      <c r="J15" s="35"/>
+      <c r="K15" s="32"/>
+      <c r="L15" s="32"/>
+      <c r="M15" s="29"/>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.4">
-      <c r="A16" s="35">
+      <c r="A16" s="26">
         <v>3</v>
       </c>
-      <c r="B16" s="22" t="s">
+      <c r="B16" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="C16" s="22" t="s">
+      <c r="C16" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="D16" s="22" t="s">
+      <c r="D16" s="27" t="s">
         <v>41</v>
       </c>
       <c r="E16" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="F16" s="22" t="s">
+      <c r="F16" s="27" t="s">
         <v>4</v>
       </c>
-      <c r="G16" s="22" t="s">
+      <c r="G16" s="27" t="s">
         <v>5</v>
       </c>
       <c r="H16" s="14" t="s">
         <v>42</v>
       </c>
-      <c r="I16" s="22" t="s">
+      <c r="I16" s="27" t="s">
         <v>7</v>
       </c>
-      <c r="J16" s="32" t="s">
+      <c r="J16" s="33" t="s">
         <v>8</v>
       </c>
-      <c r="K16" s="19">
+      <c r="K16" s="30">
         <v>244627</v>
       </c>
-      <c r="L16" s="19">
+      <c r="L16" s="30">
         <v>244628</v>
       </c>
-      <c r="M16" s="22" t="s">
+      <c r="M16" s="27" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.4">
-      <c r="A17" s="35"/>
-      <c r="B17" s="23"/>
-      <c r="C17" s="23"/>
-      <c r="D17" s="23"/>
+      <c r="A17" s="26"/>
+      <c r="B17" s="28"/>
+      <c r="C17" s="28"/>
+      <c r="D17" s="28"/>
       <c r="E17" s="5"/>
-      <c r="F17" s="23"/>
-      <c r="G17" s="23"/>
+      <c r="F17" s="28"/>
+      <c r="G17" s="28"/>
       <c r="H17" s="14"/>
-      <c r="I17" s="23"/>
-      <c r="J17" s="33"/>
-      <c r="K17" s="20"/>
-      <c r="L17" s="20"/>
-      <c r="M17" s="23"/>
+      <c r="I17" s="28"/>
+      <c r="J17" s="34"/>
+      <c r="K17" s="31"/>
+      <c r="L17" s="31"/>
+      <c r="M17" s="28"/>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.4">
-      <c r="A18" s="35"/>
-      <c r="B18" s="23"/>
-      <c r="C18" s="23"/>
-      <c r="D18" s="23"/>
+      <c r="A18" s="26"/>
+      <c r="B18" s="28"/>
+      <c r="C18" s="28"/>
+      <c r="D18" s="28"/>
       <c r="E18" s="5"/>
-      <c r="F18" s="23"/>
-      <c r="G18" s="23"/>
+      <c r="F18" s="28"/>
+      <c r="G18" s="28"/>
       <c r="H18" s="14"/>
-      <c r="I18" s="23"/>
-      <c r="J18" s="33"/>
-      <c r="K18" s="20"/>
-      <c r="L18" s="20"/>
-      <c r="M18" s="23"/>
+      <c r="I18" s="28"/>
+      <c r="J18" s="34"/>
+      <c r="K18" s="31"/>
+      <c r="L18" s="31"/>
+      <c r="M18" s="28"/>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.4">
-      <c r="A19" s="35"/>
-      <c r="B19" s="23"/>
-      <c r="C19" s="23"/>
-      <c r="D19" s="23"/>
+      <c r="A19" s="26"/>
+      <c r="B19" s="28"/>
+      <c r="C19" s="28"/>
+      <c r="D19" s="28"/>
       <c r="E19" s="5"/>
-      <c r="F19" s="23"/>
-      <c r="G19" s="23"/>
+      <c r="F19" s="28"/>
+      <c r="G19" s="28"/>
       <c r="H19" s="14"/>
-      <c r="I19" s="23"/>
-      <c r="J19" s="33"/>
-      <c r="K19" s="20"/>
-      <c r="L19" s="20"/>
-      <c r="M19" s="23"/>
+      <c r="I19" s="28"/>
+      <c r="J19" s="34"/>
+      <c r="K19" s="31"/>
+      <c r="L19" s="31"/>
+      <c r="M19" s="28"/>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.4">
-      <c r="A20" s="35"/>
-      <c r="B20" s="24"/>
-      <c r="C20" s="24"/>
-      <c r="D20" s="24"/>
+      <c r="A20" s="26"/>
+      <c r="B20" s="29"/>
+      <c r="C20" s="29"/>
+      <c r="D20" s="29"/>
       <c r="E20" s="5"/>
-      <c r="F20" s="24"/>
-      <c r="G20" s="24"/>
+      <c r="F20" s="29"/>
+      <c r="G20" s="29"/>
       <c r="H20" s="14"/>
-      <c r="I20" s="24"/>
-      <c r="J20" s="34"/>
-      <c r="K20" s="21"/>
-      <c r="L20" s="21"/>
-      <c r="M20" s="24"/>
+      <c r="I20" s="29"/>
+      <c r="J20" s="35"/>
+      <c r="K20" s="32"/>
+      <c r="L20" s="32"/>
+      <c r="M20" s="29"/>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.4">
-      <c r="A21" s="25">
+      <c r="A21" s="41">
         <v>4</v>
       </c>
-      <c r="B21" s="25" t="s">
+      <c r="B21" s="41" t="s">
         <v>44</v>
       </c>
-      <c r="C21" s="25" t="s">
+      <c r="C21" s="41" t="s">
         <v>1</v>
       </c>
-      <c r="D21" s="25" t="s">
+      <c r="D21" s="41" t="s">
         <v>47</v>
       </c>
-      <c r="E21" s="26" t="s">
+      <c r="E21" s="42" t="s">
         <v>49</v>
       </c>
-      <c r="F21" s="17" t="s">
+      <c r="F21" s="39" t="s">
         <v>4</v>
       </c>
-      <c r="G21" s="17" t="s">
+      <c r="G21" s="39" t="s">
         <v>5</v>
       </c>
-      <c r="H21" s="27"/>
-      <c r="I21" s="28" t="s">
+      <c r="H21" s="43"/>
+      <c r="I21" s="44" t="s">
         <v>7</v>
       </c>
-      <c r="J21" s="29" t="s">
+      <c r="J21" s="45" t="s">
         <v>45</v>
       </c>
-      <c r="K21" s="30">
+      <c r="K21" s="46">
         <v>46098</v>
       </c>
-      <c r="L21" s="30">
+      <c r="L21" s="46">
         <v>46099</v>
       </c>
-      <c r="M21" s="17" t="str">
+      <c r="M21" s="39" t="str">
         <f t="shared" ref="M21" si="0">(L21-K21)&amp;" วัน"</f>
         <v>1 วัน</v>
       </c>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.4">
-      <c r="A22" s="25"/>
-      <c r="B22" s="25"/>
-      <c r="C22" s="25"/>
-      <c r="D22" s="25"/>
-      <c r="E22" s="26"/>
-      <c r="F22" s="18"/>
-      <c r="G22" s="18"/>
-      <c r="H22" s="27"/>
-      <c r="I22" s="28"/>
-      <c r="J22" s="29"/>
-      <c r="K22" s="31"/>
-      <c r="L22" s="31"/>
-      <c r="M22" s="18"/>
+      <c r="A22" s="41"/>
+      <c r="B22" s="41"/>
+      <c r="C22" s="41"/>
+      <c r="D22" s="41"/>
+      <c r="E22" s="42"/>
+      <c r="F22" s="40"/>
+      <c r="G22" s="40"/>
+      <c r="H22" s="43"/>
+      <c r="I22" s="44"/>
+      <c r="J22" s="45"/>
+      <c r="K22" s="47"/>
+      <c r="L22" s="47"/>
+      <c r="M22" s="40"/>
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.4">
       <c r="A23" s="6">
@@ -1584,27 +1603,27 @@
       </c>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.4">
-      <c r="A26" s="46">
+      <c r="A26" s="17">
         <v>8</v>
       </c>
-      <c r="B26" s="46" t="s">
+      <c r="B26" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="C26" s="46" t="s">
+      <c r="C26" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="D26" s="46" t="s">
+      <c r="D26" s="17" t="s">
         <v>53</v>
       </c>
-      <c r="E26" s="47"/>
-      <c r="F26" s="46" t="s">
+      <c r="E26" s="18"/>
+      <c r="F26" s="17" t="s">
         <v>4</v>
       </c>
-      <c r="G26" s="46" t="s">
+      <c r="G26" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="H26" s="47"/>
-      <c r="I26" s="46" t="s">
+      <c r="H26" s="18"/>
+      <c r="I26" s="17" t="s">
         <v>7</v>
       </c>
       <c r="J26" s="9" t="s">
@@ -1620,25 +1639,59 @@
         <v>55</v>
       </c>
     </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.4">
+      <c r="A27" s="48">
+        <v>9</v>
+      </c>
+      <c r="B27" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="C27" s="17" t="s">
+        <v>1</v>
+      </c>
+      <c r="D27" s="48" t="s">
+        <v>56</v>
+      </c>
+      <c r="E27" s="48"/>
+      <c r="F27" s="17" t="s">
+        <v>4</v>
+      </c>
+      <c r="G27" s="12" t="s">
+        <v>5</v>
+      </c>
+      <c r="H27" s="48"/>
+      <c r="I27" s="17" t="s">
+        <v>7</v>
+      </c>
+      <c r="J27" s="49" t="s">
+        <v>57</v>
+      </c>
+      <c r="K27" s="10">
+        <v>46132</v>
+      </c>
+      <c r="L27" s="10"/>
+      <c r="M27" s="50" t="s">
+        <v>43</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="49">
-    <mergeCell ref="A1:M5"/>
-    <mergeCell ref="A6:J6"/>
-    <mergeCell ref="K6:M6"/>
-    <mergeCell ref="A8:A10"/>
-    <mergeCell ref="B8:B10"/>
-    <mergeCell ref="C8:C10"/>
-    <mergeCell ref="D8:D10"/>
-    <mergeCell ref="F8:F10"/>
-    <mergeCell ref="G8:G10"/>
-    <mergeCell ref="K11:K15"/>
-    <mergeCell ref="L11:L15"/>
-    <mergeCell ref="M11:M15"/>
-    <mergeCell ref="I8:I10"/>
-    <mergeCell ref="K8:K10"/>
-    <mergeCell ref="L8:L10"/>
-    <mergeCell ref="M8:M10"/>
-    <mergeCell ref="J8:J10"/>
+    <mergeCell ref="M21:M22"/>
+    <mergeCell ref="K16:K20"/>
+    <mergeCell ref="L16:L20"/>
+    <mergeCell ref="M16:M20"/>
+    <mergeCell ref="A21:A22"/>
+    <mergeCell ref="B21:B22"/>
+    <mergeCell ref="C21:C22"/>
+    <mergeCell ref="E21:E22"/>
+    <mergeCell ref="F21:F22"/>
+    <mergeCell ref="H21:H22"/>
+    <mergeCell ref="I21:I22"/>
+    <mergeCell ref="J21:J22"/>
+    <mergeCell ref="K21:K22"/>
+    <mergeCell ref="L21:L22"/>
+    <mergeCell ref="D21:D22"/>
+    <mergeCell ref="G21:G22"/>
     <mergeCell ref="G16:G20"/>
     <mergeCell ref="G11:G15"/>
     <mergeCell ref="I11:I15"/>
@@ -1655,22 +1708,23 @@
     <mergeCell ref="C16:C20"/>
     <mergeCell ref="D16:D20"/>
     <mergeCell ref="F16:F20"/>
-    <mergeCell ref="M21:M22"/>
-    <mergeCell ref="K16:K20"/>
-    <mergeCell ref="L16:L20"/>
-    <mergeCell ref="M16:M20"/>
-    <mergeCell ref="A21:A22"/>
-    <mergeCell ref="B21:B22"/>
-    <mergeCell ref="C21:C22"/>
-    <mergeCell ref="E21:E22"/>
-    <mergeCell ref="F21:F22"/>
-    <mergeCell ref="H21:H22"/>
-    <mergeCell ref="I21:I22"/>
-    <mergeCell ref="J21:J22"/>
-    <mergeCell ref="K21:K22"/>
-    <mergeCell ref="L21:L22"/>
-    <mergeCell ref="D21:D22"/>
-    <mergeCell ref="G21:G22"/>
+    <mergeCell ref="K11:K15"/>
+    <mergeCell ref="L11:L15"/>
+    <mergeCell ref="M11:M15"/>
+    <mergeCell ref="I8:I10"/>
+    <mergeCell ref="K8:K10"/>
+    <mergeCell ref="L8:L10"/>
+    <mergeCell ref="M8:M10"/>
+    <mergeCell ref="J8:J10"/>
+    <mergeCell ref="A1:M5"/>
+    <mergeCell ref="A6:J6"/>
+    <mergeCell ref="K6:M6"/>
+    <mergeCell ref="A8:A10"/>
+    <mergeCell ref="B8:B10"/>
+    <mergeCell ref="C8:C10"/>
+    <mergeCell ref="D8:D10"/>
+    <mergeCell ref="F8:F10"/>
+    <mergeCell ref="G8:G10"/>
   </mergeCells>
   <phoneticPr fontId="9" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>